<commit_message>
Ajout des livrables complementaires (profil, organisation, determinants, limites, SWOT, discussion, rapport de corrections)
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LmFX3Wt5gUctHSgQg4iCW4
</commit_message>
<xml_diff>
--- a/livrables-memoire-pfnl/2_Analyses_statistiques.xlsx
+++ b/livrables-memoire-pfnl/2_Analyses_statistiques.xlsx
@@ -15,6 +15,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="5. Diversité floristique" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="6. Similarité &amp; structure" sheetId="7" state="visible" r:id="rId7"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="7. Contraintes &amp; revenus" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="8. Déterminants revenu" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -24,7 +25,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="5">
+  <fonts count="9">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -53,8 +54,25 @@
       <color rgb="00FFFFFF"/>
       <sz val="10"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="000A1628"/>
+      <sz val="13"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="000A8A75"/>
+    </font>
+    <font>
+      <b val="1"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -69,6 +87,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00F1F5F9"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FDECD9"/>
       </patternFill>
     </fill>
   </fills>
@@ -98,7 +121,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -114,6 +137,14 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -5771,4 +5802,660 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E41"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="9" t="inlineStr">
+        <is>
+          <t>Facteurs déterminant le revenu PFNL total (tests non paramétriques)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="10" t="inlineStr">
+        <is>
+          <t>Facteur</t>
+        </is>
+      </c>
+      <c r="B3" s="10" t="inlineStr">
+        <is>
+          <t>Test</t>
+        </is>
+      </c>
+      <c r="C3" s="10" t="inlineStr">
+        <is>
+          <t>Statistique</t>
+        </is>
+      </c>
+      <c r="D3" s="10" t="inlineStr">
+        <is>
+          <t>p-value</t>
+        </is>
+      </c>
+      <c r="E3" s="10" t="inlineStr">
+        <is>
+          <t>Significatif ?</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="11" t="inlineStr">
+        <is>
+          <t>Ancienneté dans la collecte</t>
+        </is>
+      </c>
+      <c r="B4" s="11" t="inlineStr">
+        <is>
+          <t>Kruskal-Wallis</t>
+        </is>
+      </c>
+      <c r="C4" s="11" t="inlineStr">
+        <is>
+          <t>H = 27.23</t>
+        </is>
+      </c>
+      <c r="D4" s="11" t="inlineStr">
+        <is>
+          <t>&lt; 0,001</t>
+        </is>
+      </c>
+      <c r="E4" s="11" t="inlineStr">
+        <is>
+          <t>OUI</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="11" t="inlineStr">
+        <is>
+          <t>Nombre de PFNL collectés</t>
+        </is>
+      </c>
+      <c r="B5" s="11" t="inlineStr">
+        <is>
+          <t>Spearman</t>
+        </is>
+      </c>
+      <c r="C5" s="11" t="inlineStr">
+        <is>
+          <t>ρ = 0.524</t>
+        </is>
+      </c>
+      <c r="D5" s="11" t="inlineStr">
+        <is>
+          <t>&lt; 0,001</t>
+        </is>
+      </c>
+      <c r="E5" s="11" t="inlineStr">
+        <is>
+          <t>OUI</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="11" t="inlineStr">
+        <is>
+          <t>Groupe ethnique (Baka/Zimé)</t>
+        </is>
+      </c>
+      <c r="B6" s="11" t="inlineStr">
+        <is>
+          <t>Mann-Whitney</t>
+        </is>
+      </c>
+      <c r="C6" s="11" t="inlineStr">
+        <is>
+          <t>U = 15.5</t>
+        </is>
+      </c>
+      <c r="D6" s="11" t="n">
+        <v>0.0028</v>
+      </c>
+      <c r="E6" s="11" t="inlineStr">
+        <is>
+          <t>OUI</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="11" t="inlineStr">
+        <is>
+          <t>Appartenance au GIC</t>
+        </is>
+      </c>
+      <c r="B7" s="11" t="inlineStr">
+        <is>
+          <t>Kruskal-Wallis</t>
+        </is>
+      </c>
+      <c r="C7" s="11" t="inlineStr">
+        <is>
+          <t>H = 11.14</t>
+        </is>
+      </c>
+      <c r="D7" s="11" t="n">
+        <v>0.011</v>
+      </c>
+      <c r="E7" s="11" t="inlineStr">
+        <is>
+          <t>OUI</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="11" t="inlineStr">
+        <is>
+          <t>Lieux de collecte</t>
+        </is>
+      </c>
+      <c r="B8" s="11" t="inlineStr">
+        <is>
+          <t>Kruskal-Wallis</t>
+        </is>
+      </c>
+      <c r="C8" s="11" t="inlineStr">
+        <is>
+          <t>H = 6.0</t>
+        </is>
+      </c>
+      <c r="D8" s="11" t="n">
+        <v>0.0497</v>
+      </c>
+      <c r="E8" s="11" t="inlineStr">
+        <is>
+          <t>OUI</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>Recours à une main-d'œuvre</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>Mann-Whitney</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>U = 325.5</t>
+        </is>
+      </c>
+      <c r="D9" s="5" t="n">
+        <v>0.1147</v>
+      </c>
+      <c r="E9" s="5" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>Collecte en UFA</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>Mann-Whitney</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>U = 366.5</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="n">
+        <v>0.2943</v>
+      </c>
+      <c r="E10" s="5" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>Sexe</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>Mann-Whitney</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>U = 322.0</t>
+        </is>
+      </c>
+      <c r="D11" s="5" t="n">
+        <v>0.1332</v>
+      </c>
+      <c r="E11" s="5" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>Niveau d'instruction</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>Kruskal-Wallis</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>H = 1.74</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="n">
+        <v>0.6288</v>
+      </c>
+      <c r="E12" s="5" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>Taille du ménage</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>Kruskal-Wallis</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>H = 0.1</t>
+        </is>
+      </c>
+      <c r="D13" s="5" t="n">
+        <v>0.9923999999999999</v>
+      </c>
+      <c r="E13" s="5" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="12" t="inlineStr">
+        <is>
+          <t>Moyennes par groupe — facteurs significatifs</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="13" t="inlineStr">
+        <is>
+          <t>Ancienneté dans la collecte</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="14" t="inlineStr">
+        <is>
+          <t>Groupe</t>
+        </is>
+      </c>
+      <c r="B18" s="14" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="C18" s="14" t="inlineStr">
+        <is>
+          <t>Moyenne (FCFA)</t>
+        </is>
+      </c>
+      <c r="D18" s="14" t="inlineStr">
+        <is>
+          <t>Médiane (FCFA)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>Moins de 5 ans</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n">
+        <v>15</v>
+      </c>
+      <c r="C19" s="5" t="n">
+        <v>155700</v>
+      </c>
+      <c r="D19" s="5" t="n">
+        <v>145500</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>Entre 5 et 10 ans</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="n">
+        <v>7</v>
+      </c>
+      <c r="C20" s="5" t="n">
+        <v>776643</v>
+      </c>
+      <c r="D20" s="5" t="n">
+        <v>636500</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>Entre 10 et 15 ans</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="n">
+        <v>13</v>
+      </c>
+      <c r="C21" s="5" t="n">
+        <v>753346</v>
+      </c>
+      <c r="D21" s="5" t="n">
+        <v>774250</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>Entre 15 et 20 ans</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="n">
+        <v>9</v>
+      </c>
+      <c r="C22" s="5" t="n">
+        <v>725972</v>
+      </c>
+      <c r="D22" s="5" t="n">
+        <v>684500</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>Plus de 20 ans</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="C23" s="5" t="n">
+        <v>609625</v>
+      </c>
+      <c r="D23" s="5" t="n">
+        <v>529375</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="13" t="inlineStr">
+        <is>
+          <t>Appartenance au GIC</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="14" t="inlineStr">
+        <is>
+          <t>Groupe</t>
+        </is>
+      </c>
+      <c r="B26" s="14" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="C26" s="14" t="inlineStr">
+        <is>
+          <t>Moyenne (FCFA)</t>
+        </is>
+      </c>
+      <c r="D26" s="14" t="inlineStr">
+        <is>
+          <t>Médiane (FCFA)</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>Mpoulah Mepeh</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="n">
+        <v>17</v>
+      </c>
+      <c r="C27" s="5" t="n">
+        <v>436647</v>
+      </c>
+      <c r="D27" s="5" t="n">
+        <v>300000</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>Lumière plus</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="n">
+        <v>20</v>
+      </c>
+      <c r="C28" s="5" t="n">
+        <v>655612</v>
+      </c>
+      <c r="D28" s="5" t="n">
+        <v>578750</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t>PLACKO</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="n">
+        <v>7</v>
+      </c>
+      <c r="C29" s="5" t="n">
+        <v>815036</v>
+      </c>
+      <c r="D29" s="5" t="n">
+        <v>792500</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>Femmes Dynamiques</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="C30" s="5" t="n">
+        <v>252750</v>
+      </c>
+      <c r="D30" s="5" t="n">
+        <v>221250</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="13" t="inlineStr">
+        <is>
+          <t>Lieux de collecte</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="14" t="inlineStr">
+        <is>
+          <t>Groupe</t>
+        </is>
+      </c>
+      <c r="B33" s="14" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="C33" s="14" t="inlineStr">
+        <is>
+          <t>Moyenne (FCFA)</t>
+        </is>
+      </c>
+      <c r="D33" s="14" t="inlineStr">
+        <is>
+          <t>Médiane (FCFA)</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>Village et Forêt</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="n">
+        <v>21</v>
+      </c>
+      <c r="C34" s="5" t="n">
+        <v>651762</v>
+      </c>
+      <c r="D34" s="5" t="n">
+        <v>594250</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr">
+        <is>
+          <t>Forêt</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="n">
+        <v>22</v>
+      </c>
+      <c r="C35" s="5" t="n">
+        <v>555364</v>
+      </c>
+      <c r="D35" s="5" t="n">
+        <v>463125</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr">
+        <is>
+          <t>Village</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="n">
+        <v>7</v>
+      </c>
+      <c r="C36" s="5" t="n">
+        <v>264571</v>
+      </c>
+      <c r="D36" s="5" t="n">
+        <v>231000</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="13" t="inlineStr">
+        <is>
+          <t>Groupe ethnique (Baka/Zimé)</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="14" t="inlineStr">
+        <is>
+          <t>Groupe</t>
+        </is>
+      </c>
+      <c r="B39" s="14" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="C39" s="14" t="inlineStr">
+        <is>
+          <t>Moyenne (FCFA)</t>
+        </is>
+      </c>
+      <c r="D39" s="14" t="inlineStr">
+        <is>
+          <t>Médiane (FCFA)</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
+        <is>
+          <t>Baka</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="C40" s="5" t="n">
+        <v>100500</v>
+      </c>
+      <c r="D40" s="5" t="n">
+        <v>73500</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="5" t="inlineStr">
+        <is>
+          <t>Zimé</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="n">
+        <v>38</v>
+      </c>
+      <c r="C41" s="5" t="n">
+        <v>562618</v>
+      </c>
+      <c r="D41" s="5" t="n">
+        <v>540250</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>